<commit_message>
Fix protected route refresh session loading
</commit_message>
<xml_diff>
--- a/data/Store_Master.xlsx
+++ b/data/Store_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apparelme-my.sharepoint.com/personal/138925_appareluae_com/Documents/F&amp;B Sales Dashboard - Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="178" documentId="8_{DB8E79A2-F353-468B-8FC9-094421811B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{713A1FF7-B608-48C6-8E82-7C2A6FDD2965}"/>
+  <xr:revisionPtr revIDLastSave="182" documentId="8_{DB8E79A2-F353-468B-8FC9-094421811B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30A5487D-B248-4AFD-B977-DBFEAA310BBB}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7D4174F8-86A5-4506-B54F-CFAB4FB5A869}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="909" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="909" uniqueCount="250">
   <si>
     <t>CSC</t>
   </si>
@@ -787,6 +787,9 @@
   </si>
   <si>
     <t>Active</t>
+  </si>
+  <si>
+    <t>InActive</t>
   </si>
 </sst>
 </file>
@@ -2541,7 +2544,7 @@
         <v>231</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H48" s="1">
         <v>5101295502</v>
@@ -2570,7 +2573,7 @@
         <v>231</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H49" s="1">
         <v>5101295503</v>

</xml_diff>

<commit_message>
Build executive overview dashboard with brand cards
</commit_message>
<xml_diff>
--- a/data/Store_Master.xlsx
+++ b/data/Store_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apparelme-my.sharepoint.com/personal/138925_appareluae_com/Documents/F&amp;B Sales Dashboard - Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="183" documentId="8_{DB8E79A2-F353-468B-8FC9-094421811B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63500E51-6726-4C7F-B2B5-02CBB65DBF8D}"/>
+  <xr:revisionPtr revIDLastSave="184" documentId="8_{DB8E79A2-F353-468B-8FC9-094421811B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83C872DF-0376-41B1-91E9-3E6BC94DB5B8}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7D4174F8-86A5-4506-B54F-CFAB4FB5A869}"/>
   </bookViews>
@@ -7416,7 +7416,7 @@
         <v>234</v>
       </c>
       <c r="G216" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H216" s="1">
         <v>4101527340</v>

</xml_diff>

<commit_message>
Add dynamic filters to brand dashboard
</commit_message>
<xml_diff>
--- a/data/Store_Master.xlsx
+++ b/data/Store_Master.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apparelme-my.sharepoint.com/personal/138925_appareluae_com/Documents/F&amp;B Sales Dashboard - Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="185" documentId="8_{DB8E79A2-F353-468B-8FC9-094421811B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44929D67-3021-4040-BD91-778DC1E9CEF8}"/>
+  <xr:revisionPtr revIDLastSave="189" documentId="8_{DB8E79A2-F353-468B-8FC9-094421811B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6C3FB39-CADB-4443-9261-2E6ADDE0DB46}"/>
   <bookViews>
-    <workbookView xWindow="9670" yWindow="2110" windowWidth="11760" windowHeight="6160" xr2:uid="{7D4174F8-86A5-4506-B54F-CFAB4FB5A869}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7D4174F8-86A5-4506-B54F-CFAB4FB5A869}"/>
   </bookViews>
   <sheets>
     <sheet name="Store_Master_tbl" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Store_Master_tbl!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Store_Master_tbl!$A$1:$I$226</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -5444,7 +5444,7 @@
         <v>233</v>
       </c>
       <c r="G148" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H148" s="1">
         <v>1131916194</v>
@@ -5502,7 +5502,7 @@
         <v>233</v>
       </c>
       <c r="G150" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H150" s="1">
         <v>1132016542</v>
@@ -7716,7 +7716,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1" xr:uid="{19F24061-8C69-451B-8A49-F7670003213E}"/>
+  <autoFilter ref="A1:I226" xr:uid="{19F24061-8C69-451B-8A49-F7670003213E}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>